<commit_message>
refactor: merge noetic_bevy and noetic_runtime into noetic
A facade over a single plugin crate added a crate without adding a
boundary. The plugin crate is now `noetic`, the one games add, and it
re-exports noetic_core. Design documents, diagrams, prototype and
screenshots follow the rename.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/02_basic_design.xlsx
+++ b/docs/02_basic_design.xlsx
@@ -719,7 +719,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>0.3</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2848,6 +2848,28 @@
       <c r="D5" s="4" t="inlineStr">
         <is>
           <t>UI language decided (English, Q6); danger color decided (Q8); prototype v21.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="29" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>heryk</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>noetic_bevy and noetic_runtime merged into one crate, noetic, the crate games add; it re-exports noetic_core. C-03 kept as a removed ID.</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3152,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Noetic: open-source editor (Rust + Bevy) to create the behavior of game animals that feel alive, test it in a 2D world inside the editor and export it to a .noetic.ron file loaded by the game through the noetic_runtime crate.</t>
+          <t>Noetic: open-source editor (Rust + Bevy) to create the behavior of game animals that feel alive, test it in a 2D world inside the editor and export it to a .noetic.ron file loaded by the game through the noetic crate.</t>
         </is>
       </c>
     </row>
@@ -3559,7 +3581,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>noetic_bevy</t>
+          <t>noetic</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -3569,7 +3591,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Bevy plugin: components (NoeticAgent, WaterSource, Burrow…), systems that call noetic_core each tick, .noetic.ron AssetLoader, hot reload, animation events, debug feature (remote).</t>
+          <t>The crate games add to Cargo.toml: Bevy plugin (NoeticPlugin), components (NoeticAgent, WaterSource, Burrow…), systems that call noetic_core each tick, .noetic.ron AssetLoader, hot reload, animation events, debug feature (remote). Re-exports noetic_core with a prelude.</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -3591,27 +3613,27 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>noetic_runtime</t>
+          <t>(merged into C-02)</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Facade</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>The crate games add to Cargo.toml; re-exports core + bevy with a prelude and the NoeticPlugin.</t>
+          <t>Removed in 0.3: a facade over a single plugin crate added a crate without adding a boundary. C-02 re-exports noetic_core instead.</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>noetic_core, noetic_bevy</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>crates.io</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3638,7 +3660,7 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>bevy, bevy_feathers, noetic_runtime</t>
+          <t>bevy, bevy_feathers, noetic</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -3747,7 +3769,7 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>noetic_runtime</t>
+          <t>noetic</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -3771,7 +3793,7 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>noetic_runtime + bevy_remote</t>
+          <t>noetic + bevy_remote</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -4028,7 +4050,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Noetic does not implement 3D navigation; adapter trait in noetic_bevy.</t>
+          <t>Noetic does not implement 3D navigation; adapter trait in noetic.</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs: drop the Japanese names from the workbook covers
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/02_basic_design.xlsx
+++ b/docs/02_basic_design.xlsx
@@ -681,11 +681,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>基本設計書</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -707,7 +703,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Basic Design (基本設計書)</t>
+          <t>Basic Design</t>
         </is>
       </c>
     </row>
@@ -719,7 +715,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.4</t>
         </is>
       </c>
     </row>
@@ -779,7 +775,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Requirements Definition (要件定義) · External Design (外部設計書) · Detailed Design (詳細設計書, to be written)</t>
+          <t>Requirements Definition · External Design · Detailed Design (to be written)</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2870,6 +2866,28 @@
       <c r="D6" s="4" t="inlineStr">
         <is>
           <t>noetic_bevy and noetic_runtime merged into one crate, noetic, the crate games add; it re-exports noetic_core. C-03 kept as a removed ID.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>heryk</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Japanese names removed; the documents are in English only.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: let the game move the animals and share one agent pipeline
</commit_message>
<xml_diff>
--- a/docs/02_basic_design.xlsx
+++ b/docs/02_basic_design.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>0.7</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
+    <row r="6" ht="68" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>IF-03</t>
@@ -1213,7 +1213,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Animation events</t>
+          <t>Animation, alarm and death events</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>NoeticAnimEvent { entity, event: String, looping: bool } at step start/end; game maps to its AnimationGraph using animation_clips.</t>
+          <t>NoeticAnimEvent { entity, event: String, clip: Option&lt;String&gt;, looping: bool } at step start/end, clip taken from the species animation_clips; the game plays it on its AnimationGraph. NoeticAlarm { entity, kind } for game audio; NoeticDied { entity }.</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="29" customHeight="1">
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>IF-04</t>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>WaterSource, Burrow, Bush, Tree, Food, Cover, Mud, NoiseEvent, NoeticPlayer — read by perception and step targets.</t>
+          <t>WaterSource, Burrow, Bush, Tree, Food, Cover, Mud, NoiseEmitter, NoeticPlayer — marker zones with a radius, read by perception and step targets; unmarked ground is open.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1269,7 +1269,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
+    <row r="8" ht="55" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>IF-05</t>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Navigation adapter</t>
+          <t>Movement intent</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1287,12 +1287,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Rust trait</t>
+          <t>Bevy components</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>NoeticNavigator { fn path(from, to) -&gt; Option&lt;Path&gt; } implemented by the game with its navmesh crate; default straight-line for 2D/simple games.</t>
+          <t>MoveIntent { target, gait, speed, gaze } written by Noetic every fixed step; the game moves the Transform with its own navigation. Optional MoveFailed marker when the target is unreachable.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -2144,7 +2144,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="29" customHeight="1">
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>NFR-03</t>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>noetic_core depends only on serde/ron/rand_core; unit tests per PRC step.</t>
+          <t>noetic_core depends only on the crates listed in Internal Design › 2 Workspace (serde, ron, rand_core + rand_pcg, thiserror, glam, smallvec), never on Bevy; unit tests per PRC step.</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Perception and choice at a configurable rate (default 10 Hz), movement every frame; spatial grid for neighbours; criterion benches in CI. Animal-count target: open (Q2).</t>
+          <t>Perception and choice at a configurable rate (default 10 Hz), movement intent every fixed step (60 Hz); spatial grid for neighbours; criterion benches in CI. Animal-count target: open (Q2).</t>
         </is>
       </c>
     </row>
@@ -2558,12 +2558,12 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Navigation from existing crates</t>
+          <t>Movement belongs to the game</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Adapter IF-05.</t>
+          <t>Noetic publishes MoveIntent (IF-05); no navigation crate.</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2888,6 +2888,72 @@
       <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Japanese names removed; the documents are in English only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>heryk</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>The game moves the animals: Noetic publishes a movement intent (IF-05 MoveIntent, replaces the NoeticNavigator adapter); C-02, T-07, F-607, PRC-15 and CON-03 updated. World components are marker zones with a radius (F-704, IF-04).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>heryk</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>One agent pipeline: PRC-03…10 think at think_hz, PRC-11…15 act every fixed step; what an agent does to others is queued as an Effect and applied by the new PRC-17 (PRC-09, PRC-13, PRC-14 updated).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="55" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>heryk</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Coherence review: PRC-10 noise is a factor; Need gets Safety and Company; IF-03 carries clip, NoeticAlarm and NoeticDied; IF-04 NoiseEmitter; C-01 and NFR-03 list the noetic_core crates of Internal Design 2; NFR-04 movement intent every fixed step; source is Requirements Definition v0.4.</t>
         </is>
       </c>
     </row>
@@ -3206,7 +3272,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Requirements Definition v0.2 (FR-xxx / NFR-xx) and clickable prototype v21 (English UI).</t>
+          <t>Requirements Definition v0.4 (FR-xxx / NFR-xx) and clickable prototype v21 (English UI).</t>
         </is>
       </c>
     </row>
@@ -3582,7 +3648,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>serde, ron, rand_core (seeded PRNG)</t>
+          <t>serde, ron, rand_core + rand_pcg (seeded PRNG), thiserror, glam, smallvec</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -3591,7 +3657,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="55" customHeight="1">
+    <row r="28" ht="68" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>C-02</t>
@@ -3609,7 +3675,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>The crate games add to Cargo.toml: Bevy plugin (NoeticPlugin), components (NoeticAgent, WaterSource, Burrow…), systems that call noetic_core each tick, .noetic.ron AssetLoader, hot reload, animation events, debug feature (remote). Re-exports noetic_core with a prelude.</t>
+          <t>The crate games add to Cargo.toml: Bevy plugin (NoeticPlugin), components (NoeticAgent, WaterSource, Burrow…), systems that call noetic_core each tick, .noetic.ron AssetLoader, hot reload, animation events, movement intents, debug feature (remote). Re-exports noetic_core with a prelude.</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -4050,7 +4116,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="29" customHeight="1">
+    <row r="10" ht="42" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>T-07</t>
@@ -4063,17 +4129,17 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Existing navmesh crate</t>
+          <t>None: the game moves the animals</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Noetic does not implement 3D navigation; adapter trait in noetic.</t>
+          <t>The game moves the animals from MoveIntent (IF-05) with its own navigation; Noetic needs no navigation crate.</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Crate to choose</t>
+          <t>Chosen by the game</t>
         </is>
       </c>
     </row>
@@ -5707,7 +5773,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16" customHeight="1">
+    <row r="36" ht="42" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
           <t>F-607</t>
@@ -5730,7 +5796,7 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Hop/zigzag/flight/perch; terrain speed; obstacles.</t>
+          <t>Movement intent: target, gait (hop/zigzag/flight/perch), speed, gaze; the game moves the body. Editor: simple mover with terrain speed and obstacles.</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -5942,7 +6008,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="16" customHeight="1">
+    <row r="41" ht="29" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
           <t>F-704</t>
@@ -5965,7 +6031,7 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>WaterSource, Burrow, Cover, Food… read by perception.</t>
+          <t>WaterSource, Burrow, Cover, Food, Mud… marker zones with a radius, read by perception and step targets; unmarked ground is open.</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
@@ -6146,7 +6212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6180,7 +6246,7 @@
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>5.1 Simulation tick (noetic_core::tick, fixed order, per agent unless noted)</t>
+          <t>5.1 Simulation tick (fixed order, per agent unless noted: PRC-03…10 think at think_hz, PRC-11…15 act every fixed step, PRC-17 applies effects after every agent)</t>
         </is>
       </c>
     </row>
@@ -6535,7 +6601,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Alarm reactions (thump, tail, chirp) raise fear of nearby agents, including other species.</t>
+          <t>Alarm reactions (thump, tail, chirp) queue an Effect; PRC-17 raises the fear of nearby agents, including other species.</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -6572,7 +6638,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>When idle: score = curve(need) × weight × routine factor + noise; pick best.</t>
+          <t>When idle: score = curve(need) × weight × routine factor × (1 ± noise); pick best.</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -6665,7 +6731,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="29" customHeight="1">
+    <row r="18" ht="42" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>PRC-13</t>
@@ -6683,7 +6749,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Approach rival, scuffle, apply damage; the other fights back or flees; cooldown on failure.</t>
+          <t>Approach rival, scuffle; damage and the challenge are queued as Effects; the rival fights back or flees in its own think; cooldown on failure.</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -6702,7 +6768,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16" customHeight="1">
+    <row r="19" ht="29" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>PRC-14</t>
@@ -6720,7 +6786,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Leave marks at frequency; decay marks (world-level).</t>
+          <t>Leave marks at frequency (queued as an Effect); decay marks (world-level).</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -6739,7 +6805,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="29" customHeight="1">
+    <row r="20" ht="42" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>PRC-15</t>
@@ -6752,17 +6818,17 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>target, terrain</t>
+          <t>target, gait, limp</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Move with species gait; terrain speed factor; obstacles; navmesh in game.</t>
+          <t>Write the movement intent (target, gait, speed, gaze); the game moves the body and Sync reads the position back. Editor: simple mover with terrain speed and obstacles.</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>position</t>
+          <t>MoveIntent</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -6813,304 +6879,341 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+    <row r="22" ht="42" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>PRC-17</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Apply effects</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>effects of every agent</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>World-level, after every agent acted: sort effects by (source id, seq); alarms raise the fear of agents in their radius, damage and challenges reach their target, marks are stored.</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>fear, health, marks</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>F-604</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>FR-504, 506, 507</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>5.2 Editor flows</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Flow</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>Trigger</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E25" s="7" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>F-ID</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>Screen</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="29" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="26" ht="29" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>PRC-21</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Export species</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Export .ron</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Compile graph → species brain (first, reactions, choose, activities) → serialize RON with schema_version → show/save.</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>.noetic.ron</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>F-701</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>DLG-02</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="42" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>PRC-22</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Import species</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Import</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>Read text → parse RON → check schema_version and migrate → validate (weights, ids, DAG) → resolve name clash → build graph.</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>new species</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>F-702</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>DLG-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="29" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>PRC-23</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Hot reload (game)</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>File changed</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>AssetLoader reloads → agents keep state, brain swapped at next decision.</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>updated behavior</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>F-703</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
         </is>
       </c>
     </row>
     <row r="28" ht="29" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>PRC-24</t>
+          <t>PRC-23</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Reaction sandbox</t>
+          <t>Hot reload (game)</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Any change on SCR-14</t>
+          <t>File changed</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Clone peers + minimal world; set stimulus; fixed seed; run tick for N s; record segments.</t>
+          <t>AssetLoader reloads → agents keep state, brain swapped at next decision.</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>result list</t>
+          <t>updated behavior</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>F-504</t>
+          <t>F-703</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>SCR-14</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="29" ht="29" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
+          <t>PRC-24</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Reaction sandbox</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Any change on SCR-14</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Clone peers + minimal world; set stimulus; fixed seed; run tick for N s; record segments.</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>result list</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>F-504</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>SCR-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="29" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
           <t>PRC-25</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>Remote debug</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Connect</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>BRP request every 250 ms → list agents → selected agent state → show in Details panel.</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>live view</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>F-705</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>DLG-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>PRC-26</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Undo</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Ctrl+Z / toast</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>Pop command from stack and apply its inverse.</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>previous state</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>F-102</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>All</t>
         </is>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
+          <t>PRC-26</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Undo</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Ctrl+Z / toast</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Pop command from stack and apply its inverse.</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>previous state</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>F-102</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
           <t>PRC-27</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Autosave</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>Every change (debounced 2 s)</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>Write project file atomically (temp + rename).</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>project saved</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>F-103</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -8315,7 +8418,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Hunger | Thirst | Fatigue | Fear | Boredom | Mark | Fight | Sing | Heat | Calm</t>
+          <t>Hunger | Thirst | Fatigue | Fear | Safety | Company | Boredom | Mark | Fight | Sing | Heat | Calm</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: save the individuals and make the documents agree with each other
</commit_message>
<xml_diff>
--- a/docs/02_basic_design.xlsx
+++ b/docs/02_basic_design.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t xml:space="preserve">0.11</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Requirements Definition · External Design · Detailed Design (to be written)</t>
+          <t xml:space="preserve">Requirements Definition · External Design · Internal Design · Detailed Design</t>
         </is>
       </c>
     </row>
@@ -891,11 +891,11 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Folders, species, activities (shared), presets, world (ENT-09), settings, UI state. Autosaved atomically.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="29" customHeight="1">
+          <t xml:space="preserve">Folders, species, activities (shared), presets, world (ENT-09), individuals (ENT-08: species, name, seed, position, traits, quirks, locked), settings, UI state. Autosaved atomically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>FMT-03</t>
@@ -932,23 +932,23 @@
     <row r="9" ht="225" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>NoeticSpecies(
+          <t xml:space="preserve">NoeticSpecies(
   schema_version: 1,
   species: "rabbit", color: "#D8D2C4",
-  locomotion: Ground(hop: true, speed: 2.4, flee_speed: 9.0),
+  locomotion: (kind: Ground, hop: true, speed: 2.4, flee_speed: 9.0),
   group: Solitary, shelter: Burrow, routine: Crepuscular,
   senses: (vision: 30.0, angle: 340.0, hearing: 45.0, smell: 20.0, night_vision: 0.55),
   needs: (hunger_per_h: 25.0, thirst_per_h: 30.0, fatigue_per_h: 12.0, fear_threshold: 60.0),
   health: (max: 30.0, pain_resist: 0.2, heal_per_h: 4.0, limp_below: 0.4),
   personality: (base: {"fear": 78, ...}, variation: {"fear": 18, ...}),
-  scent_marks: [(kind: Urine, meaning: Safe, every_min: 40.0, lasts_h: 48.0)],
+  scent_marks: (enabled: true, kinds: [Urine, Chin, Latrine], meaning: [Safe], every_min: 40.0, lasts_h: 48.0),
   brain: (
     threat: (first: [("freeze", 60), ("flee", 40)],
              reactions: {"freeze": (do: Freeze(secs: 2.0), next: [("thump", 70), ("flee", 30)]), ...}),
     choose: (noise: 0.15, options: ["graze", "drink", "rest", "watch", "groom", "dig", "mark"]),
   ),
-  activities: {"graze": (need: Hunger, curve: Accelerating, weight: 1.0, steps: [...])},
-  animation_clips: {"graze": "Rabbit_Eat", "drink": "Rabbit_Drink"},
+  activities: {"graze": (need: Hunger, curve: Accelerating, weight: 1.0, steps: [...]), ...},
+  animation_clips: {"graze": "Rabbit_Eat", "watch": "Rabbit_Stand", "drink": "Rabbit_Drink"},
 )</t>
         </is>
       </c>
@@ -1006,7 +1006,7 @@
       <c r="D13" s="4" t="inlineStr"/>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Unknown id → line number</t>
+          <t xml:space="preserve">Unknown id → message naming the id</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>NoeticAnimEvent { entity, event: String, clip: Option&lt;String&gt;, looping: bool } at step start/end, clip taken from the species animation_clips; the game plays it on its AnimationGraph. NoeticAlarm { entity, kind } for game audio; NoeticDied { entity }.</t>
+          <t xml:space="preserve">NoeticAnimEvent { entity, event: String, clip: Option&lt;String&gt;, looping: bool } at step start (looping is true for steps and for Freeze and Hide, false for one-shot reactions such as Alarm and Charge), clip taken from the species animation_clips; the game plays it on its AnimationGraph. NoeticAlarm { entity, kind } for game audio; NoeticDied { entity }.</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>WaterSource, Burrow, Bush, Tree, Food, Cover, Mud, NoiseEmitter, NoeticPlayer — marker zones with a radius, read by perception and step targets; unmarked ground is open.</t>
+          <t xml:space="preserve">WaterSource, Burrow, Bush, Tree, Food, Cover, Mud — marker zones with a radius; NoiseEmitter (radius, ttl) and NoeticPlayer (movement state, cover). Read by perception and step targets; unmarked ground is open.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Editor simulation calls noetic_core::tick; no editor-only behavior code.</t>
+          <t xml:space="preserve">Editor simulation calls noetic::sim::tick (noetic_core, re-exported); no editor-only behavior code.</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>All parsing returns Result; editor shows messages (MSG-013); runtime logs and skips invalid species.</t>
+          <t xml:space="preserve">All parsing returns Result; editor shows messages (MSG-013); runtime logs the error and leaves that species' agents idle (EP-02).</t>
         </is>
       </c>
     </row>
@@ -2723,7 +2723,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Event only vs. despawn policy.</t>
+          <t xml:space="preserve">Decided: event only. Noetic emits NoeticDied and stops processing the agent; the game decides whether the body stays, despawns or respawns.</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2954,6 +2954,94 @@
       <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Coherence review: PRC-10 noise is a factor; Need gets Safety and Company; IF-03 carries clip, NoeticAlarm and NoeticDied; IF-04 NoiseEmitter; C-01 and NFR-03 list the noetic_core crates of Internal Design 2; NFR-04 movement intent every fixed step; source is Requirements Definition v0.4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>heryk</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Individuals are saved: the edits of ENT-08 (species, name, seed, position, traits, quirks, lock) go in FMT-02 with ENT-11, needs, fear, health and memory start fresh; F-103 covers FR-402 and FR-404. FR-115 in F-201, FR-114 in F-203, FR-201 and FR-213 in F-304 (Map, camera and layers). Source is Requirements Definition v0.5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="68" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.9</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-17</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">heryk</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Review against the other documents: PRC-16 Events runs after PRC-17 Apply, so a death from damage goes out the same step; the Crate column says noetic, not bevy (F-607, F-703…705); C-05 removed, the extension traits live in noetic_core::ext; T-05 fixed to rand_pcg; C-04 lists the editor crates; IF-03 events at step start; IF-04 tells the zones from NoiseEmitter and NoeticPlayer; CRUD F-103 creates agents; Q7 decided; cover lists the Internal Design; source is Requirements Definition v0.6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="68" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.10</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-17</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">heryk</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each document checked against itself: every Need has its own rate (needs.rates) and Fear is no longer a Need; locomotion is a struct with a kind; scent_marks is one struct (enabled, kinds, meaning, every_min, lasts_h); the FMT-01 example follows them and marks its shortened activity map; the editor depends on plain noetic (C-04, ENV-01); F-203 also runs in core (PRC-11); PRC-13 queues effects, the rival answers in its own act; PRC-15 names noetic::sync; PRC-17 traces to F-604…606; CRUD gets F-405 and F-702 updates the project; ENT-02/03/05/06 live in FMT-01 and FMT-02; Agent attributes list what the editor saves, and the field is locked; ENT-11 includes UI state; source is Requirements Definition v0.7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="68" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.11</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-17</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">heryk</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Needs follow the prototype: hunger, thirst and fatigue keep their rates, heat and sing follow the hour, safety and company the place, the rest are driving values (PRC-04); Fear is a Need again and Curiosity joins (Need); PRC-07 uses fear_trait / 100; PRC-10, 13, 15, 17 cite F-608, FR-508 and IF-05; IF-03 says when looping is true; F-405 spawns animals when asked; CRUD gets F-502 and F-306; the Agent attributes mark what FMT-02 saves (locked); scent marks default to off; V-02, NFR-02, NFR-12 match the Internal Design; the editor lists slotmap; the FMT-01 example shows watch in animation_clips; source is Requirements Definition v0.8.</t>
         </is>
       </c>
     </row>
@@ -3272,7 +3360,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Requirements Definition v0.4 (FR-xxx / NFR-xx) and clickable prototype v21 (English UI).</t>
+          <t xml:space="preserve">Requirements Definition v0.8 (FR-xxx / NFR-xx) and clickable prototype v21 (English UI).</t>
         </is>
       </c>
     </row>
@@ -3744,7 +3832,7 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>bevy, bevy_feathers, noetic</t>
+          <t xml:space="preserve">bevy (ui, feathers), noetic, arboard, rfd, ureq, slotmap</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -3761,27 +3849,27 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>noetic_ext (optional)</t>
+          <t xml:space="preserve">(merged into C-01)</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Extension API</t>
+          <t xml:space="preserve">—</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Traits NoeticAction, NoeticCondition, NoeticSensor, UtilityCurve; registration so code-defined nodes appear in the editor. May live inside noetic_core.</t>
+          <t xml:space="preserve">Removed in 0.9: the extension traits live in the noetic_core::ext module (Internal Design MOD-006), so games still add only noetic.</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>noetic_core</t>
+          <t xml:space="preserve">—</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>crates.io</t>
+          <t xml:space="preserve">—</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3917,7 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>noetic_editor + noetic_core</t>
+          <t xml:space="preserve">noetic_editor + noetic</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -4075,7 +4163,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Seeded PRNG per agent (e.g. rand_pcg / rand_chacha)</t>
+          <t xml:space="preserve">Seeded PRNG per agent: Pcg32 (rand_pcg) behind noetic_core::rng</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -4085,7 +4173,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>To decide in DD</t>
+          <t xml:space="preserve">Fixed</t>
         </is>
       </c>
     </row>
@@ -4433,7 +4521,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Autosave and load of the editor project file (FMT-02).</t>
+          <t>Autosave and load of the editor project file (FMT-02), individuals included.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -4448,7 +4536,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>NFR-05</t>
+          <t>FR-402, 404, NFR-05</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -4480,7 +4568,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Root, Threat, Reaction, Choose-activity and Activity blocks; connect/disconnect; connection rules; cycle check; loose-block warning.</t>
+          <t>Root, Threat, Reaction, Choose-activity and Activity blocks; connect/disconnect; connection rules; cycle check; loose-block warning; zoom, fit and pan.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -4495,7 +4583,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>FR-101–104</t>
+          <t>FR-101–104, 115</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -4574,12 +4662,12 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Step subgraph: Start + ordered steps (type, min–max duration, animation event).</t>
+          <t xml:space="preserve">Step subgraph: Start + ordered steps (type, min–max duration, animation event); warning when the activity is shared by several species; the runtime runs the steps (PRC-11).</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>editor</t>
+          <t xml:space="preserve">editor + core</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -4589,7 +4677,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>FR-107, 108</t>
+          <t>FR-107, 108, 114</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -4880,7 +4968,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="29" customHeight="1">
+    <row r="17" ht="42" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>F-304</t>
@@ -4898,12 +4986,12 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Camera and layers</t>
+          <t>Map, camera and layers</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Zoom, pan, minimap, debug layers, wind.</t>
+          <t>Colored 240 × 150 m top-down map (river, ponds, mud, woods, hills, rocks, burrows, tall grass, clover) in a neutral interface; zoom, pan, minimap, debug layers, wind.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -4918,7 +5006,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>FR-202, 207, 208</t>
+          <t>FR-201, 202, 207, 208, 213</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -5232,7 +5320,7 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Blank or from template.</t>
+          <t xml:space="preserve">Blank or from template; spawns 4 animals when asked.</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -5801,7 +5889,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>core + bevy</t>
+          <t xml:space="preserve">core + noetic</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -5989,7 +6077,7 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>bevy</t>
+          <t xml:space="preserve">noetic</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -6036,7 +6124,7 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>bevy</t>
+          <t xml:space="preserve">noetic</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -6083,7 +6171,7 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>bevy + editor</t>
+          <t xml:space="preserve">noetic + editor</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -6246,7 +6334,7 @@
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>5.1 Simulation tick (fixed order, per agent unless noted: PRC-03…10 think at think_hz, PRC-11…15 act every fixed step, PRC-17 applies effects after every agent)</t>
+          <t xml:space="preserve">5.1 Simulation tick (fixed order, per agent unless noted: PRC-03…10 think at think_hz, PRC-11…15 act every fixed step, PRC-17 applies effects after every agent, then PRC-16 sends the events)</t>
         </is>
       </c>
     </row>
@@ -6416,7 +6504,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Increase needs by rate × dt; current activity lowers its need.</t>
+          <t xml:space="preserve">Hunger, thirst and fatigue rise by their rate × dt_h (dt_h = dt / secs_per_game_hour); heat and sing follow the hour, safety the distance to the shelter, company the distance to the group; the other driving values are computed when choosing (Detailed ALG-02). The current activity lowers its need (PRC-11).</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -6527,7 +6615,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>fear += best × (0.4 + fear_trait × 1.2) × 60 × dt; decay near own safe marks; pain adds fear.</t>
+          <t xml:space="preserve">fear += best × (0.4 + fear_trait / 100 × 1.2) × 60 × dt (dt in seconds); decay near own safe marks; pain adds fear.</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -6648,7 +6736,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>F-204</t>
+          <t xml:space="preserve">F-204, F-608</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -6749,12 +6837,12 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Approach rival, scuffle; damage and the challenge are queued as Effects; the rival fights back or flees in its own think; cooldown on failure.</t>
+          <t xml:space="preserve">Approach rival, scuffle; damage and the challenge are queued as Effects; the rival fights back or flees in its own act; cooldown on failure.</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>health, fear</t>
+          <t xml:space="preserve">effects (damage, challenge)</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -6764,7 +6852,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>FR-507</t>
+          <t xml:space="preserve">FR-507, 508</t>
         </is>
       </c>
     </row>
@@ -6823,7 +6911,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Write the movement intent (target, gait, speed, gaze); the game moves the body and Sync reads the position back. Editor: simple mover with terrain speed and obstacles.</t>
+          <t xml:space="preserve">Write the movement intent (target, gait, speed, gaze); the game moves the body and noetic::sync (IF-05) reads the position back. Editor: simple mover with terrain speed and obstacles.</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -6842,77 +6930,77 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16" customHeight="1">
+    <row r="21" ht="42" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>PRC-16</t>
+          <t xml:space="preserve">PRC-17</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Events out</t>
+          <t xml:space="preserve">Apply effects</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>state changes</t>
+          <t xml:space="preserve">effects of every agent</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Emit events for the host (animation, sound, death).</t>
+          <t xml:space="preserve">World-level, after every agent acted: sort effects by (source id, seq); alarms raise the fear of agents in their radius, damage and challenges reach their target, marks are stored.</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>events[]</t>
+          <t xml:space="preserve">fear, health, marks</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>F-703</t>
+          <t xml:space="preserve">F-604, F-605, F-606</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>FR-603</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="42" customHeight="1">
+          <t xml:space="preserve">FR-504, 506, 507, 508</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="29" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>PRC-17</t>
+          <t xml:space="preserve">PRC-16</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Apply effects</t>
+          <t xml:space="preserve">Events out</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>effects of every agent</t>
+          <t xml:space="preserve">state changes</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>World-level, after every agent acted: sort effects by (source id, seq); alarms raise the fear of agents in their radius, damage and challenges reach their target, marks are stored.</t>
+          <t xml:space="preserve">Emit events for the host (animation, sound, death), after PRC-17 so a death from damage goes out in the same step.</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>fear, health, marks</t>
+          <t xml:space="preserve">events[]</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>F-604</t>
+          <t xml:space="preserve">F-703</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>FR-504, 506, 507</t>
+          <t xml:space="preserve">FR-603</t>
         </is>
       </c>
     </row>
@@ -7235,7 +7323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7358,7 +7446,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>FMT-01</t>
+          <t xml:space="preserve">FMT-01 / FMT-02</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr"/>
@@ -7387,7 +7475,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>FMT-01</t>
+          <t xml:space="preserve">FMT-01 / FMT-02</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr"/>
@@ -7449,7 +7537,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>FMT-01</t>
+          <t xml:space="preserve">FMT-01 / FMT-02</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr"/>
@@ -7478,7 +7566,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>FMT-01</t>
+          <t xml:space="preserve">FMT-01 / FMT-02</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr"/>
@@ -7522,7 +7610,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="29" customHeight="1">
+    <row r="13" ht="42" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>ENT-08</t>
@@ -7540,7 +7628,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>memory only</t>
+          <t>memory; edits in FMT-02</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -7551,7 +7639,7 @@
       <c r="F13" s="4" t="inlineStr"/>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>One living animal: seed, traits, quirks, needs, fear, health, memory, state.</t>
+          <t xml:space="preserve">One living animal: seed, traits, quirks, needs, fear, health, memory, state. The editor saves species, name, seed, position, traits, quirks, locked; the rest starts fresh on load.</t>
         </is>
       </c>
     </row>
@@ -7650,7 +7738,7 @@
       <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Folders, species, activities, presets, world, settings.</t>
+          <t xml:space="preserve">Folders, species, activities, presets, world, individuals, settings, UI state.</t>
         </is>
       </c>
     </row>
@@ -7818,7 +7906,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>enum Ground{hop,speed,flee_speed} | Bird{…}</t>
+          <t xml:space="preserve">struct { kind: Ground | Bird, hop, speed, flee_speed }</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -7984,7 +8072,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>hunger/thirst/fatigue per hour 0–60; fear_threshold 0–100</t>
+          <t xml:space="preserve">hunger/thirst/fatigue per hour 0–60; fear_threshold 0–100; the other needs follow their driver (PRC-04)</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr"/>
@@ -8107,17 +8195,17 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Vec&lt;{kind, meaning, every_min, lasts_h}&gt;</t>
+          <t xml:space="preserve">struct { enabled, kinds, meaning, every_min, lasts_h }</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>kind: Urine|Chin|Latrine|Scrape|Antler|Body; meaning: Safe|Territory|Alert</t>
+          <t xml:space="preserve">kinds ⊆ Urine|Chin|Latrine|Scrape|Antler|Body; meaning ⊆ Safe|Territory|Alert; every_min 5–240; lasts_h 1–168</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t xml:space="preserve">enabled: false (templates turn it on)</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -8418,7 +8506,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Hunger | Thirst | Fatigue | Fear | Safety | Company | Boredom | Mark | Fight | Sing | Heat | Calm</t>
+          <t xml:space="preserve">Hunger | Thirst | Fatigue | Fear | Safety | Company | Curiosity | Boredom | Mark | Fight | Sing | Heat | Calm</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr"/>
@@ -8648,319 +8736,379 @@
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>Determinism.</t>
+          <t xml:space="preserve">Determinism. Saved in FMT-02.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Agent</t>
+          <t xml:space="preserve">Agent</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>traits</t>
+          <t xml:space="preserve">species</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Map&lt;trait, u8&gt;</t>
+          <t xml:space="preserve">SpeciesId</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>0–100</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>from species</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G50" s="4" t="inlineStr"/>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saved in FMT-02.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="16" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Agent</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">String</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1–40 chars</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">from the species name pool</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saved in FMT-02.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Agent</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vec2</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inside the world</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near the shelter</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saved in FMT-02.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="16" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Agent</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quirks</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vec&lt;String&gt;</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0–5</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1–2 from the species pool</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saved in FMT-02.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="16" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
           <t>Agent</t>
         </is>
       </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>traits</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Map&lt;trait, u8&gt;</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>0–100</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>from species</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saved in FMT-02.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="16" customHeight="1">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>locked</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>bool</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr"/>
-      <c r="E51" s="4" t="inlineStr">
+      <c r="D55" s="4" t="inlineStr"/>
+      <c r="E55" s="4" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="F51" s="4" t="inlineStr">
+      <c r="F55" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G51" s="4" t="inlineStr"/>
-    </row>
-    <row r="52" ht="29" customHeight="1">
-      <c r="A52" s="4" t="inlineStr">
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saved in FMT-02.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="29" customHeight="1">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>Agent</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>needs / fear / health</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>f32</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
+      <c r="D56" s="4" t="inlineStr">
         <is>
           <t>0–100 / 0–100 / 0–max</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr"/>
-      <c r="F52" s="4" t="inlineStr">
+      <c r="E56" s="4" t="inlineStr"/>
+      <c r="F56" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G52" s="4" t="inlineStr"/>
-    </row>
-    <row r="53" ht="55" customHeight="1">
-      <c r="A53" s="4" t="inlineStr">
+      <c r="G56" s="4" t="inlineStr"/>
+    </row>
+    <row r="57" ht="55" customHeight="1">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>Agent</t>
         </is>
       </c>
-      <c r="B53" s="4" t="inlineStr">
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>memory</t>
         </is>
       </c>
-      <c r="C53" s="4" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>struct</t>
         </is>
       </c>
-      <c r="D53" s="4" t="inlineStr">
+      <c r="D57" s="4" t="inlineStr">
         <is>
           <t>habituation, scare spots, water, shelter, marks (with age)</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr"/>
-      <c r="F53" s="4" t="inlineStr">
+      <c r="E57" s="4" t="inlineStr"/>
+      <c r="F57" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G53" s="4" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="12" t="inlineStr">
+      <c r="G57" s="4" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr">
         <is>
           <t>6.3 CRUD matrix (C create · R read · U update · D delete)</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="7" t="inlineStr">
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="7" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="B56" s="7" t="inlineStr">
+      <c r="B60" s="7" t="inlineStr">
         <is>
           <t>Species</t>
         </is>
       </c>
-      <c r="C56" s="7" t="inlineStr">
+      <c r="C60" s="7" t="inlineStr">
         <is>
           <t>Activity</t>
         </is>
       </c>
-      <c r="D56" s="7" t="inlineStr">
+      <c r="D60" s="7" t="inlineStr">
         <is>
           <t>Preset</t>
         </is>
       </c>
-      <c r="E56" s="7" t="inlineStr">
+      <c r="E60" s="7" t="inlineStr">
         <is>
           <t>Agent</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
+      <c r="F60" s="7" t="inlineStr">
         <is>
           <t>World</t>
         </is>
       </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="G60" s="7" t="inlineStr">
         <is>
           <t>ScentMark</t>
         </is>
       </c>
-      <c r="H56" s="7" t="inlineStr">
+      <c r="H60" s="7" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="4" t="inlineStr">
+    <row r="61" ht="16" customHeight="1">
+      <c r="A61" s="4" t="inlineStr">
         <is>
           <t>F-101 Tree</t>
         </is>
       </c>
-      <c r="B57" s="4" t="inlineStr">
+      <c r="B61" s="4" t="inlineStr">
         <is>
           <t>CRUD</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>CRUD</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr"/>
-      <c r="E57" s="4" t="inlineStr"/>
-      <c r="F57" s="4" t="inlineStr"/>
-      <c r="G57" s="4" t="inlineStr"/>
-      <c r="H57" s="4" t="inlineStr">
+      <c r="D61" s="4" t="inlineStr"/>
+      <c r="E61" s="4" t="inlineStr"/>
+      <c r="F61" s="4" t="inlineStr"/>
+      <c r="G61" s="4" t="inlineStr"/>
+      <c r="H61" s="4" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="29" customHeight="1">
-      <c r="A58" s="4" t="inlineStr">
+    <row r="62" ht="29" customHeight="1">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>F-201 Species graph</t>
         </is>
       </c>
-      <c r="B58" s="4" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>RU</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr"/>
-      <c r="E58" s="4" t="inlineStr"/>
-      <c r="F58" s="4" t="inlineStr"/>
-      <c r="G58" s="4" t="inlineStr"/>
-      <c r="H58" s="4" t="inlineStr"/>
-    </row>
-    <row r="59" ht="29" customHeight="1">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>F-203 Activity steps</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="inlineStr"/>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
-      <c r="D59" s="4" t="inlineStr"/>
-      <c r="E59" s="4" t="inlineStr"/>
-      <c r="F59" s="4" t="inlineStr"/>
-      <c r="G59" s="4" t="inlineStr"/>
-      <c r="H59" s="4" t="inlineStr"/>
-    </row>
-    <row r="60" ht="29" customHeight="1">
-      <c r="A60" s="4" t="inlineStr">
-        <is>
-          <t>F-303 Stimuli / spawn</t>
-        </is>
-      </c>
-      <c r="B60" s="4" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="inlineStr"/>
-      <c r="D60" s="4" t="inlineStr"/>
-      <c r="E60" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F60" s="4" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="G60" s="4" t="inlineStr"/>
-      <c r="H60" s="4" t="inlineStr"/>
-    </row>
-    <row r="61" ht="29" customHeight="1">
-      <c r="A61" s="4" t="inlineStr">
-        <is>
-          <t>F-305 Terrain editing</t>
-        </is>
-      </c>
-      <c r="B61" s="4" t="inlineStr"/>
-      <c r="C61" s="4" t="inlineStr"/>
-      <c r="D61" s="4" t="inlineStr"/>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>CRUD</t>
-        </is>
-      </c>
-      <c r="G61" s="4" t="inlineStr"/>
-      <c r="H61" s="4" t="inlineStr"/>
-    </row>
-    <row r="62" ht="42" customHeight="1">
-      <c r="A62" s="4" t="inlineStr">
-        <is>
-          <t>F-401–404 Species pages</t>
-        </is>
-      </c>
-      <c r="B62" s="4" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
-      <c r="C62" s="4" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="D62" s="4" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E62" s="4" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="D62" s="4" t="inlineStr"/>
+      <c r="E62" s="4" t="inlineStr"/>
       <c r="F62" s="4" t="inlineStr"/>
       <c r="G62" s="4" t="inlineStr"/>
       <c r="H62" s="4" t="inlineStr"/>
@@ -8968,21 +9116,17 @@
     <row r="63" ht="29" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>F-402 Presets</t>
+          <t>F-203 Activity steps</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr"/>
-      <c r="C63" s="4" t="inlineStr"/>
-      <c r="D63" s="4" t="inlineStr">
-        <is>
-          <t>CRD</t>
-        </is>
-      </c>
-      <c r="E63" s="4" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr"/>
+      <c r="E63" s="4" t="inlineStr"/>
       <c r="F63" s="4" t="inlineStr"/>
       <c r="G63" s="4" t="inlineStr"/>
       <c r="H63" s="4" t="inlineStr"/>
@@ -8990,7 +9134,7 @@
     <row r="64" ht="29" customHeight="1">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>F-501 Personality</t>
+          <t>F-303 Stimuli / spawn</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -8999,124 +9143,132 @@
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr"/>
-      <c r="D64" s="4" t="inlineStr">
+      <c r="D64" s="4" t="inlineStr"/>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="E64" s="4" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
-      <c r="F64" s="4" t="inlineStr"/>
       <c r="G64" s="4" t="inlineStr"/>
       <c r="H64" s="4" t="inlineStr"/>
     </row>
     <row r="65" ht="29" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>F-504 Sandbox</t>
-        </is>
-      </c>
-      <c r="B65" s="4" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="C65" s="4" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+          <t>F-305 Terrain editing</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr"/>
+      <c r="C65" s="4" t="inlineStr"/>
       <c r="D65" s="4" t="inlineStr"/>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>R (copies)</t>
+          <t>R</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>CRUD</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr"/>
       <c r="H65" s="4" t="inlineStr"/>
     </row>
-    <row r="66" ht="29" customHeight="1">
+    <row r="66" ht="42" customHeight="1">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>F-6xx Runtime tick</t>
+          <t>F-401–404 Species pages</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
           <t>R</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr">
+      <c r="D66" s="4" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="D66" s="4" t="inlineStr"/>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>RU</t>
-        </is>
-      </c>
-      <c r="F66" s="4" t="inlineStr">
-        <is>
           <t>R</t>
         </is>
       </c>
-      <c r="G66" s="4" t="inlineStr">
-        <is>
-          <t>CRUD</t>
-        </is>
-      </c>
+      <c r="F66" s="4" t="inlineStr"/>
+      <c r="G66" s="4" t="inlineStr"/>
       <c r="H66" s="4" t="inlineStr"/>
     </row>
-    <row r="67" ht="29" customHeight="1">
+    <row r="67" ht="16" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>F-701 Export</t>
+          <t xml:space="preserve">F-405 New species</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>R</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="D67" s="4" t="inlineStr"/>
-      <c r="E67" s="4" t="inlineStr"/>
-      <c r="F67" s="4" t="inlineStr"/>
-      <c r="G67" s="4" t="inlineStr"/>
-      <c r="H67" s="4" t="inlineStr"/>
+          <t xml:space="preserve">R</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">U</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="29" customHeight="1">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>F-702 Import</t>
-        </is>
-      </c>
-      <c r="B68" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D68" s="4" t="inlineStr"/>
-      <c r="E68" s="4" t="inlineStr"/>
+          <t>F-402 Presets</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr"/>
+      <c r="C68" s="4" t="inlineStr"/>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>CRD</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
       <c r="F68" s="4" t="inlineStr"/>
       <c r="G68" s="4" t="inlineStr"/>
       <c r="H68" s="4" t="inlineStr"/>
@@ -9124,32 +9276,258 @@
     <row r="69" ht="29" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
         <is>
+          <t>F-501 Personality</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr"/>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr"/>
+      <c r="G69" s="4" t="inlineStr"/>
+      <c r="H69" s="4" t="inlineStr"/>
+    </row>
+    <row r="70" ht="16" customHeight="1">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F-502 Quirks</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">U</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="16" customHeight="1">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F-306 Quick tests</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">U</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="29" customHeight="1">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>F-504 Sandbox</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr"/>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>R (copies)</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G72" s="4" t="inlineStr"/>
+      <c r="H72" s="4" t="inlineStr"/>
+    </row>
+    <row r="73" ht="29" customHeight="1">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>F-6xx Runtime tick</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr"/>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>CRUD</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr"/>
+    </row>
+    <row r="74" ht="29" customHeight="1">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>F-701 Export</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr"/>
+      <c r="E74" s="4" t="inlineStr"/>
+      <c r="F74" s="4" t="inlineStr"/>
+      <c r="G74" s="4" t="inlineStr"/>
+      <c r="H74" s="4" t="inlineStr"/>
+    </row>
+    <row r="75" ht="29" customHeight="1">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>F-702 Import</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr"/>
+      <c r="E75" s="4" t="inlineStr"/>
+      <c r="F75" s="4" t="inlineStr"/>
+      <c r="G75" s="4" t="inlineStr"/>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">U</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="29" customHeight="1">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
           <t>F-103 Save / load</t>
         </is>
       </c>
-      <c r="B69" s="4" t="inlineStr">
+      <c r="B76" s="4" t="inlineStr">
         <is>
           <t>CR</t>
         </is>
       </c>
-      <c r="C69" s="4" t="inlineStr">
+      <c r="C76" s="4" t="inlineStr">
         <is>
           <t>CR</t>
         </is>
       </c>
-      <c r="D69" s="4" t="inlineStr">
+      <c r="D76" s="4" t="inlineStr">
         <is>
           <t>CR</t>
         </is>
       </c>
-      <c r="E69" s="4" t="inlineStr"/>
-      <c r="F69" s="4" t="inlineStr">
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
         <is>
           <t>CR</t>
         </is>
       </c>
-      <c r="G69" s="4" t="inlineStr"/>
-      <c r="H69" s="4" t="inlineStr">
+      <c r="G76" s="4" t="inlineStr"/>
+      <c r="H76" s="4" t="inlineStr">
         <is>
           <t>CRU</t>
         </is>

</xml_diff>

<commit_message>
feat: add the seeded Rng and weighted_pick to noetic_core
</commit_message>
<xml_diff>
--- a/docs/02_basic_design.xlsx
+++ b/docs/02_basic_design.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.11</t>
+          <t xml:space="preserve">0.12</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>noetic_core depends only on the crates listed in Internal Design › 2 Workspace (serde, ron, rand_core + rand_pcg, thiserror, glam, smallvec), never on Bevy; unit tests per PRC step.</t>
+          <t>noetic_core depends only on the crates listed in Internal Design › 2 Workspace (serde, ron, rand + rand_pcg, thiserror, glam, smallvec), never on Bevy; unit tests per PRC step.</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3042,6 +3042,28 @@
       <c r="D14" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Needs follow the prototype: hunger, thirst and fatigue keep their rates, heat and sing follow the hour, safety and company the place, the rest are driving values (PRC-04); Fear is a Need again and Curiosity joins (Need); PRC-07 uses fear_trait / 100; PRC-10, 13, 15, 17 cite F-608, FR-508 and IF-05; IF-03 says when looping is true; F-405 spawns animals when asked; CRUD gets F-502 and F-306; the Agent attributes mark what FMT-02 saves (locked); scent marks default to off; V-02, NFR-02, NFR-12 match the Internal Design; the editor lists slotmap; the FMT-01 example shows watch in animation_clips; source is Requirements Definition v0.8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="68" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.12</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-19</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">heryk</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">noetic_core samples through rand (no default features, so no thread_rng) instead of rand_core; Pcg32 behind noetic_core::rng is unchanged (T-05).</t>
         </is>
       </c>
     </row>
@@ -3736,7 +3758,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>serde, ron, rand_core + rand_pcg (seeded PRNG), thiserror, glam, smallvec</t>
+          <t>serde, ron, rand + rand_pcg (seeded PRNG), thiserror, glam, smallvec</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">

</xml_diff>

<commit_message>
feat: add Need, Curve, Routine, NeedRates and Needs to noetic_core
</commit_message>
<xml_diff>
--- a/docs/02_basic_design.xlsx
+++ b/docs/02_basic_design.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.12</t>
+          <t xml:space="preserve">0.13</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>noetic_core depends only on the crates listed in Internal Design › 2 Workspace (serde, ron, rand + rand_pcg, thiserror, glam, smallvec), never on Bevy; unit tests per PRC step.</t>
+          <t>noetic_core depends only on the crates listed in Internal Design › 2 Workspace (serde, ron, rand + rand_pcg, thiserror, glam, smallvec, enum-map), never on Bevy; unit tests per PRC step.</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3064,6 +3064,28 @@
       <c r="D15" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">noetic_core samples through rand (no default features, so no thread_rng) instead of rand_core; Pcg32 behind noetic_core::rng is unchanged (T-05).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="68" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.13</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-19</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">heryk</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">noetic_core adds enum-map for the needs of an animal, one value per Need; a well-known crate is preferred to code written by hand (CONTRIBUTING › Dependencies).</t>
         </is>
       </c>
     </row>
@@ -3758,7 +3780,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>serde, ron, rand + rand_pcg (seeded PRNG), thiserror, glam, smallvec</t>
+          <t>serde, ron, rand + rand_pcg (seeded PRNG), thiserror, glam, smallvec, enum-map</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">

</xml_diff>

<commit_message>
feat: add GoToTarget, StepKind and Step, and give activities their steps
</commit_message>
<xml_diff>
--- a/docs/02_basic_design.xlsx
+++ b/docs/02_basic_design.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.13</t>
+          <t xml:space="preserve">0.14</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3086,6 +3086,28 @@
       <c r="D16" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">noetic_core adds enum-map for the needs of an animal, one value per Need; a well-known crate is preferred to code written by hand (CONTRIBUTING › Dependencies).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="68" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.14</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-19</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">heryk</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The target of a GoTo step is a GoToTarget (Food, Water, Shelter, MarkSpot, Mud, Rival, Perch), the destinations of the prototype's go-to steps.</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8696,7 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Wander | GoTo(target) | Sniff | Watch | Eat | Drink | Rest | Groom | Dig | Mark | Wallow | Rub | Fight | Sing | Perch | Custom</t>
+          <t>Wander | GoTo(GoToTarget: Food | Water | Shelter | MarkSpot | Mud | Rival | Perch) | Sniff | Watch | Eat | Drink | Rest | Groom | Dig | Mark | Wallow | Rub | Fight | Sing | Perch | Custom</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr"/>

</xml_diff>